<commit_message>
data update, wokring code, results figure created
</commit_message>
<xml_diff>
--- a/scm_input_cleaned.xlsx
+++ b/scm_input_cleaned.xlsx
@@ -1,29 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5611d695511771a1/Desktop/Repositories/scm_model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="525" documentId="8_{69118542-9163-4E18-BF71-86AAA6BFC266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A2DBF90-A9BA-4883-A216-4AFD2263B6C8}"/>
+  <xr:revisionPtr revIDLastSave="599" documentId="8_{69118542-9163-4E18-BF71-86AAA6BFC266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7FA5C165-ABC6-4551-971D-EF91E34A1543}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="6825" windowWidth="29040" windowHeight="17520" xr2:uid="{D3628906-A666-41FC-B4DD-112A108B04C0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="4" xr2:uid="{D3628906-A666-41FC-B4DD-112A108B04C0}"/>
   </bookViews>
   <sheets>
     <sheet name="timeseries" sheetId="1" r:id="rId1"/>
     <sheet name="sink_blocks" sheetId="2" r:id="rId2"/>
     <sheet name="economic_cc_tech" sheetId="3" r:id="rId3"/>
     <sheet name="cc_tech" sheetId="8" r:id="rId4"/>
-    <sheet name="ng_flows" sheetId="4" r:id="rId5"/>
-    <sheet name="distances" sheetId="6" r:id="rId6"/>
-    <sheet name="economic_transport" sheetId="7" r:id="rId7"/>
+    <sheet name="cc_commited_cap" sheetId="9" r:id="rId5"/>
+    <sheet name="ng_flows" sheetId="4" r:id="rId6"/>
+    <sheet name="distances" sheetId="6" r:id="rId7"/>
+    <sheet name="economic_transport" sheetId="7" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">ng_flows!$D$1:$D$217</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">sink_blocks!$A$1:$A$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">ng_flows!$D$1:$D$217</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">sink_blocks!$C$1:$C$60</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -250,7 +251,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1022" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1023" uniqueCount="160">
   <si>
     <t>year</t>
   </si>
@@ -516,36 +517,6 @@
     <t>ir_cap</t>
   </si>
   <si>
-    <t>3,500,000</t>
-  </si>
-  <si>
-    <t>2,500,000</t>
-  </si>
-  <si>
-    <t>2,000,000</t>
-  </si>
-  <si>
-    <t>3,000,000</t>
-  </si>
-  <si>
-    <t>8,000,000</t>
-  </si>
-  <si>
-    <t>1,000,000</t>
-  </si>
-  <si>
-    <t>500,000</t>
-  </si>
-  <si>
-    <t>1,500,000</t>
-  </si>
-  <si>
-    <t>4,000,000</t>
-  </si>
-  <si>
-    <t>6,000,000</t>
-  </si>
-  <si>
     <t>Industry_cement</t>
   </si>
   <si>
@@ -703,6 +674,63 @@
   </si>
   <si>
     <t>ENTSOE CO2 Price Trajectory</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>EU|psc_cement</t>
+  </si>
+  <si>
+    <t>EU|psc_chemicals</t>
+  </si>
+  <si>
+    <t>EU|psc_iron_steel</t>
+  </si>
+  <si>
+    <t>EU|psc_otherindustry</t>
+  </si>
+  <si>
+    <t>EU|psc_power</t>
+  </si>
+  <si>
+    <t>EU|psc_refining</t>
+  </si>
+  <si>
+    <t>NO|psc_cement</t>
+  </si>
+  <si>
+    <t>NO|psc_chemicals</t>
+  </si>
+  <si>
+    <t>NO|psc_iron_steel</t>
+  </si>
+  <si>
+    <t>NO|psc_otherindustry</t>
+  </si>
+  <si>
+    <t>NO|psc_power</t>
+  </si>
+  <si>
+    <t>NO|psc_refining</t>
+  </si>
+  <si>
+    <t>UK|psc_cement</t>
+  </si>
+  <si>
+    <t>UK|psc_chemicals</t>
+  </si>
+  <si>
+    <t>UK|psc_iron_steel</t>
+  </si>
+  <si>
+    <t>UK|psc_otherindustry</t>
+  </si>
+  <si>
+    <t>UK|psc_power</t>
+  </si>
+  <si>
+    <t>UK|psc_refining</t>
   </si>
 </sst>
 </file>
@@ -767,7 +795,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -777,6 +805,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -796,7 +836,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -816,6 +856,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Komma" xfId="1" builtinId="3"/>
@@ -1272,7 +1318,7 @@
         <v>21</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>51</v>
@@ -2447,7 +2493,7 @@
         <v>8</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="F27" s="4" t="s">
         <v>10</v>
@@ -2476,7 +2522,7 @@
         <v>11</v>
       </c>
       <c r="E28" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="F28" t="s">
         <v>12</v>
@@ -2515,6 +2561,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA852480-4336-48A0-952D-1FD697CF57B6}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:O60"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2531,7 +2578,7 @@
         <v>24</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>25</v>
@@ -2570,12 +2617,12 @@
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>38</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="C2">
         <v>2</v>
@@ -2594,16 +2641,16 @@
         <v>207000000</v>
       </c>
       <c r="H2">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I2">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J2">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K2">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L2">
         <v>6</v>
@@ -2623,7 +2670,7 @@
         <v>38</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -2641,16 +2688,16 @@
         <v>2400000</v>
       </c>
       <c r="H3">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I3">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J3">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K3">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L3">
         <v>6</v>
@@ -2665,12 +2712,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>38</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="C4">
         <v>2</v>
@@ -2689,16 +2736,16 @@
         <v>160000000</v>
       </c>
       <c r="H4">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I4">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J4">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K4">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L4">
         <v>6</v>
@@ -2718,7 +2765,7 @@
         <v>38</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -2737,16 +2784,16 @@
         <v>400000000</v>
       </c>
       <c r="H5">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I5">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J5">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K5">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L5">
         <v>6</v>
@@ -2766,7 +2813,7 @@
         <v>38</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -2785,16 +2832,16 @@
         <v>67000000</v>
       </c>
       <c r="H6">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I6">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J6">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K6">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L6">
         <v>6</v>
@@ -2814,7 +2861,7 @@
         <v>38</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -2833,16 +2880,16 @@
         <v>43000000</v>
       </c>
       <c r="H7">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I7">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J7">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K7">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L7">
         <v>6</v>
@@ -2862,7 +2909,7 @@
         <v>38</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -2881,16 +2928,16 @@
         <v>100000000</v>
       </c>
       <c r="H8">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I8">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J8">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K8">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L8">
         <v>6</v>
@@ -2910,7 +2957,7 @@
         <v>38</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -2928,16 +2975,16 @@
         <v>37000000</v>
       </c>
       <c r="H9">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I9">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J9">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K9">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L9">
         <v>6</v>
@@ -2976,16 +3023,16 @@
         <v>50000000</v>
       </c>
       <c r="H10">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I10">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J10">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K10">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L10">
         <v>6</v>
@@ -3024,16 +3071,16 @@
         <v>30000000</v>
       </c>
       <c r="H11">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I11">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J11">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K11">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L11">
         <v>6</v>
@@ -3072,16 +3119,16 @@
         <v>20000000</v>
       </c>
       <c r="H12">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I12">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J12">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K12">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L12">
         <v>6</v>
@@ -3101,7 +3148,7 @@
         <v>38</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="C13">
         <v>1</v>
@@ -3119,16 +3166,16 @@
         <v>2000000</v>
       </c>
       <c r="H13">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I13">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J13">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K13">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L13">
         <v>6</v>
@@ -3143,12 +3190,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>38</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="C14">
         <v>2</v>
@@ -3167,16 +3214,16 @@
         <v>498000000</v>
       </c>
       <c r="H14">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I14">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J14">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K14">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L14">
         <v>6</v>
@@ -3196,7 +3243,7 @@
         <v>38</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="C15">
         <v>1</v>
@@ -3215,16 +3262,16 @@
         <v>32000000</v>
       </c>
       <c r="H15">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I15">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J15">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K15">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L15">
         <v>6</v>
@@ -3239,12 +3286,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
         <v>38</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="C16">
         <v>2</v>
@@ -3263,16 +3310,16 @@
         <v>34200000</v>
       </c>
       <c r="H16">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I16">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J16">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K16">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L16">
         <v>6</v>
@@ -3292,7 +3339,7 @@
         <v>38</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="C17">
         <v>1</v>
@@ -3311,16 +3358,16 @@
         <v>360000000</v>
       </c>
       <c r="H17">
-        <v>20</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="I17">
-        <v>19.2</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="J17">
-        <v>18.43</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="K17">
-        <v>17.690000000000001</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="L17">
         <v>6</v>
@@ -3340,7 +3387,7 @@
         <v>38</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -3359,16 +3406,16 @@
         <v>250000000</v>
       </c>
       <c r="H18">
-        <v>20</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="I18">
-        <v>19.2</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="J18">
-        <v>18.43</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="K18">
-        <v>17.690000000000001</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="L18">
         <v>6</v>
@@ -3407,16 +3454,16 @@
         <v>54000000</v>
       </c>
       <c r="H19">
-        <v>20</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="I19">
-        <v>19.2</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="J19">
-        <v>18.43</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="K19">
-        <v>17.690000000000001</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="L19">
         <v>6</v>
@@ -3436,7 +3483,7 @@
         <v>38</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="C20">
         <v>1</v>
@@ -3455,16 +3502,16 @@
         <v>122999999.99999999</v>
       </c>
       <c r="H20">
-        <v>20</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="I20">
-        <v>19.2</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="J20">
-        <v>18.43</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="K20">
-        <v>17.690000000000001</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="L20">
         <v>6</v>
@@ -3503,16 +3550,16 @@
         <v>12000000</v>
       </c>
       <c r="H21">
-        <v>10</v>
+        <v>1.7</v>
       </c>
       <c r="I21">
-        <v>9.6</v>
+        <v>1.7</v>
       </c>
       <c r="J21">
-        <v>9.2200000000000006</v>
+        <v>1.7</v>
       </c>
       <c r="K21">
-        <v>8.85</v>
+        <v>1.7</v>
       </c>
       <c r="L21">
         <v>4</v>
@@ -3532,7 +3579,7 @@
         <v>38</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="C22">
         <v>1</v>
@@ -3551,16 +3598,16 @@
         <v>12000000</v>
       </c>
       <c r="H22">
-        <v>10</v>
+        <v>1.7</v>
       </c>
       <c r="I22">
-        <v>9.6</v>
+        <v>1.7</v>
       </c>
       <c r="J22">
-        <v>9.2200000000000006</v>
+        <v>1.7</v>
       </c>
       <c r="K22">
-        <v>8.85</v>
+        <v>1.7</v>
       </c>
       <c r="L22">
         <v>4</v>
@@ -3580,7 +3627,7 @@
         <v>38</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="C23">
         <v>1</v>
@@ -3599,16 +3646,16 @@
         <v>20000000</v>
       </c>
       <c r="H23">
-        <v>10</v>
+        <v>1.7</v>
       </c>
       <c r="I23">
-        <v>9.6</v>
+        <v>1.7</v>
       </c>
       <c r="J23">
-        <v>9.2200000000000006</v>
+        <v>1.7</v>
       </c>
       <c r="K23">
-        <v>8.85</v>
+        <v>1.7</v>
       </c>
       <c r="L23">
         <v>4</v>
@@ -3628,7 +3675,7 @@
         <v>38</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="C24">
         <v>1</v>
@@ -3647,16 +3694,16 @@
         <v>20000000</v>
       </c>
       <c r="H24">
-        <v>10</v>
+        <v>1.7</v>
       </c>
       <c r="I24">
-        <v>9.6</v>
+        <v>1.7</v>
       </c>
       <c r="J24">
-        <v>9.2200000000000006</v>
+        <v>1.7</v>
       </c>
       <c r="K24">
-        <v>8.85</v>
+        <v>1.7</v>
       </c>
       <c r="L24">
         <v>4</v>
@@ -3676,7 +3723,7 @@
         <v>38</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="C25">
         <v>1</v>
@@ -3695,16 +3742,16 @@
         <v>10000000</v>
       </c>
       <c r="H25">
-        <v>12</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="I25">
-        <v>11.52</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="J25">
-        <v>11.06</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="K25">
-        <v>10.62</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="L25">
         <v>4</v>
@@ -3719,12 +3766,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
         <v>38</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="C26">
         <v>2</v>
@@ -3742,16 +3789,16 @@
         <v>90000000</v>
       </c>
       <c r="H26">
-        <v>12</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="I26">
-        <v>11.52</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="J26">
-        <v>11.06</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="K26">
-        <v>10.62</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="L26">
         <v>4</v>
@@ -3790,16 +3837,16 @@
         <v>15770000</v>
       </c>
       <c r="H27">
-        <v>12</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="I27">
-        <v>11.52</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="J27">
-        <v>11.06</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="K27">
-        <v>10.62</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="L27">
         <v>4</v>
@@ -3838,16 +3885,16 @@
         <v>15800000</v>
       </c>
       <c r="H28">
-        <v>12</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="I28">
-        <v>11.52</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="J28">
-        <v>11.06</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="K28">
-        <v>10.62</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="L28">
         <v>4</v>
@@ -3886,16 +3933,16 @@
         <v>5600000</v>
       </c>
       <c r="H29">
-        <v>12</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="I29">
-        <v>11.52</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="J29">
-        <v>11.06</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="K29">
-        <v>10.62</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="L29">
         <v>4</v>
@@ -3933,16 +3980,16 @@
         <v>16000000</v>
       </c>
       <c r="H30">
-        <v>12</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="I30">
-        <v>11.52</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="J30">
-        <v>11.06</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="K30">
-        <v>10.62</v>
+        <v>2.2250000000000001</v>
       </c>
       <c r="L30">
         <v>4</v>
@@ -3962,7 +4009,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="C31">
         <v>1</v>
@@ -3981,16 +4028,16 @@
         <v>42750000</v>
       </c>
       <c r="H31">
-        <v>20</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="I31">
-        <v>19.2</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="J31">
-        <v>18.43</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="K31">
-        <v>17.690000000000001</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="L31">
         <v>6</v>
@@ -4005,12 +4052,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>29</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="C32">
         <v>2</v>
@@ -4029,16 +4076,16 @@
         <v>150000000</v>
       </c>
       <c r="H32">
-        <v>20</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="I32">
-        <v>19.2</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="J32">
-        <v>18.43</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="K32">
-        <v>17.690000000000001</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="L32">
         <v>6</v>
@@ -4058,7 +4105,7 @@
         <v>29</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="C33">
         <v>1</v>
@@ -4076,16 +4123,16 @@
         <v>37500000</v>
       </c>
       <c r="H33">
-        <v>20</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="I33">
-        <v>19.2</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="J33">
-        <v>18.43</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="K33">
-        <v>17.690000000000001</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="L33">
         <v>6</v>
@@ -4100,12 +4147,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>29</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="C34">
         <v>2</v>
@@ -4124,16 +4171,16 @@
         <v>87500000</v>
       </c>
       <c r="H34">
-        <v>20</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="I34">
-        <v>19.2</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="J34">
-        <v>18.43</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="K34">
-        <v>17.690000000000001</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="L34">
         <v>6</v>
@@ -4153,7 +4200,7 @@
         <v>29</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="C35">
         <v>1</v>
@@ -4172,16 +4219,16 @@
         <v>500000000</v>
       </c>
       <c r="H35">
-        <v>20</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="I35">
-        <v>19.2</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="J35">
-        <v>18.43</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="K35">
-        <v>17.690000000000001</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="L35">
         <v>6</v>
@@ -4201,7 +4248,7 @@
         <v>29</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="C36">
         <v>1</v>
@@ -4220,16 +4267,16 @@
         <v>200000000</v>
       </c>
       <c r="H36">
-        <v>20</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="I36">
-        <v>19.2</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="J36">
-        <v>18.43</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="K36">
-        <v>17.690000000000001</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="L36">
         <v>6</v>
@@ -4249,7 +4296,7 @@
         <v>29</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="C37">
         <v>1</v>
@@ -4268,16 +4315,16 @@
         <v>300000000</v>
       </c>
       <c r="H37">
-        <v>20</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="I37">
-        <v>19.2</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="J37">
-        <v>18.43</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="K37">
-        <v>17.690000000000001</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="L37">
         <v>6</v>
@@ -4297,7 +4344,7 @@
         <v>29</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="C38">
         <v>1</v>
@@ -4315,16 +4362,16 @@
         <v>100000000</v>
       </c>
       <c r="H38">
-        <v>20</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="I38">
-        <v>19.2</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="J38">
-        <v>18.43</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="K38">
-        <v>17.690000000000001</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="L38">
         <v>6</v>
@@ -4344,7 +4391,7 @@
         <v>29</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="C39">
         <v>1</v>
@@ -4363,16 +4410,16 @@
         <v>120000000</v>
       </c>
       <c r="H39">
-        <v>20</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="I39">
-        <v>19.2</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="J39">
-        <v>18.43</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="K39">
-        <v>17.690000000000001</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="L39">
         <v>6</v>
@@ -4392,7 +4439,7 @@
         <v>30</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="C40">
         <v>1</v>
@@ -4411,16 +4458,16 @@
         <v>330000000</v>
       </c>
       <c r="H40">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I40">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J40">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K40">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L40">
         <v>6</v>
@@ -4440,7 +4487,7 @@
         <v>30</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="C41">
         <v>1</v>
@@ -4459,16 +4506,16 @@
         <v>150000000</v>
       </c>
       <c r="H41">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I41">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J41">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K41">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L41">
         <v>6</v>
@@ -4488,7 +4535,7 @@
         <v>30</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="C42">
         <v>1</v>
@@ -4507,16 +4554,16 @@
         <v>135000000</v>
       </c>
       <c r="H42">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I42">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J42">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K42">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L42">
         <v>6</v>
@@ -4531,12 +4578,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>30</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="C43">
         <v>2</v>
@@ -4555,16 +4602,16 @@
         <v>55000000</v>
       </c>
       <c r="H43">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I43">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J43">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K43">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L43">
         <v>6</v>
@@ -4584,7 +4631,7 @@
         <v>30</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="C44">
         <v>1</v>
@@ -4603,16 +4650,16 @@
         <v>72000000</v>
       </c>
       <c r="H44">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I44">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J44">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K44">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L44">
         <v>6</v>
@@ -4627,12 +4674,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>30</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="C45">
         <v>2</v>
@@ -4651,16 +4698,16 @@
         <v>128000000</v>
       </c>
       <c r="H45">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I45">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J45">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K45">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L45">
         <v>6</v>
@@ -4675,12 +4722,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>30</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="C46">
         <v>3</v>
@@ -4699,16 +4746,16 @@
         <v>100000000</v>
       </c>
       <c r="H46">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I46">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J46">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K46">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L46">
         <v>6</v>
@@ -4728,7 +4775,7 @@
         <v>30</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="C47">
         <v>1</v>
@@ -4747,16 +4794,16 @@
         <v>100000000</v>
       </c>
       <c r="H47">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I47">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J47">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K47">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L47">
         <v>6</v>
@@ -4776,7 +4823,7 @@
         <v>30</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="C48">
         <v>1</v>
@@ -4795,16 +4842,16 @@
         <v>1000000000</v>
       </c>
       <c r="H48">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I48">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J48">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K48">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L48">
         <v>6</v>
@@ -4824,7 +4871,7 @@
         <v>30</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="C49">
         <v>1</v>
@@ -4843,16 +4890,16 @@
         <v>60000000</v>
       </c>
       <c r="H49">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I49">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J49">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K49">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L49">
         <v>6</v>
@@ -4867,12 +4914,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>30</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="C50">
         <v>2</v>
@@ -4891,16 +4938,16 @@
         <v>297500000</v>
       </c>
       <c r="H50">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I50">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J50">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K50">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L50">
         <v>6</v>
@@ -4915,12 +4962,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>30</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="C51">
         <v>3</v>
@@ -4939,16 +4986,16 @@
         <v>330000000</v>
       </c>
       <c r="H51">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I51">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J51">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K51">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L51">
         <v>6</v>
@@ -4968,7 +5015,7 @@
         <v>30</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="C52">
         <v>1</v>
@@ -4987,16 +5034,16 @@
         <v>30000000</v>
       </c>
       <c r="H52">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I52">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J52">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K52">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L52">
         <v>6</v>
@@ -5011,12 +5058,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>30</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="C53">
         <v>2</v>
@@ -5034,16 +5081,16 @@
         <v>150000000</v>
       </c>
       <c r="H53">
-        <v>14</v>
+        <v>2.4</v>
       </c>
       <c r="I53">
-        <v>13.44</v>
+        <v>2.4</v>
       </c>
       <c r="J53">
-        <v>12.9</v>
+        <v>2.4</v>
       </c>
       <c r="K53">
-        <v>12.39</v>
+        <v>2.4</v>
       </c>
       <c r="L53">
         <v>6</v>
@@ -5063,7 +5110,7 @@
         <v>30</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="C54">
         <v>1</v>
@@ -5082,16 +5129,16 @@
         <v>200000000</v>
       </c>
       <c r="H54">
-        <v>20</v>
+        <v>2.4</v>
       </c>
       <c r="I54">
-        <v>19.2</v>
+        <v>2.4</v>
       </c>
       <c r="J54">
-        <v>18.43</v>
+        <v>2.4</v>
       </c>
       <c r="K54">
-        <v>17.690000000000001</v>
+        <v>2.4</v>
       </c>
       <c r="L54">
         <v>6</v>
@@ -5111,7 +5158,7 @@
         <v>30</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="C55">
         <v>1</v>
@@ -5130,16 +5177,16 @@
         <v>90000000</v>
       </c>
       <c r="H55">
-        <v>20</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="I55">
-        <v>19.2</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="J55">
-        <v>18.43</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="K55">
-        <v>17.690000000000001</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="L55">
         <v>6</v>
@@ -5159,7 +5206,7 @@
         <v>30</v>
       </c>
       <c r="B56" s="8" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="C56">
         <v>1</v>
@@ -5178,16 +5225,16 @@
         <v>90000000</v>
       </c>
       <c r="H56">
-        <v>20</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="I56">
-        <v>19.2</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="J56">
-        <v>18.43</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="K56">
-        <v>17.690000000000001</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="L56">
         <v>6</v>
@@ -5207,7 +5254,7 @@
         <v>30</v>
       </c>
       <c r="B57" s="8" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="C57">
         <v>1</v>
@@ -5226,16 +5273,16 @@
         <v>100000000</v>
       </c>
       <c r="H57">
-        <v>20</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="I57">
-        <v>19.2</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="J57">
-        <v>18.43</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="K57">
-        <v>17.690000000000001</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="L57">
         <v>6</v>
@@ -5250,12 +5297,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>30</v>
       </c>
       <c r="B58" s="8" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="C58">
         <v>2</v>
@@ -5273,16 +5320,16 @@
         <v>150000000</v>
       </c>
       <c r="H58">
-        <v>20</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="I58">
-        <v>19.2</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="J58">
-        <v>18.43</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="K58">
-        <v>17.690000000000001</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="L58">
         <v>6</v>
@@ -5302,7 +5349,7 @@
         <v>30</v>
       </c>
       <c r="B59" s="8" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C59">
         <v>1</v>
@@ -5321,16 +5368,16 @@
         <v>80000000</v>
       </c>
       <c r="H59">
-        <v>20</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="I59">
-        <v>19.2</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="J59">
-        <v>18.43</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="K59">
-        <v>17.690000000000001</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="L59">
         <v>6</v>
@@ -5345,12 +5392,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>30</v>
       </c>
       <c r="B60" s="8" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C60">
         <v>2</v>
@@ -5369,16 +5416,16 @@
         <v>285000000</v>
       </c>
       <c r="H60">
-        <v>20</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="I60">
-        <v>19.2</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="J60">
-        <v>18.43</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="K60">
-        <v>17.690000000000001</v>
+        <v>4.2249999999999996</v>
       </c>
       <c r="L60">
         <v>6</v>
@@ -5394,6 +5441,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="C1:C60" xr:uid="{EA852480-4336-48A0-952D-1FD697CF57B6}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="1"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -5406,6 +5460,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="20.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -5431,16 +5486,16 @@
         <v>50</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>58</v>
@@ -5452,21 +5507,21 @@
         <v>60</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B2" t="s">
         <v>61</v>
@@ -5475,31 +5530,27 @@
         <v>57</v>
       </c>
       <c r="D2" s="6">
-        <v>143</v>
+        <v>370.07860257398664</v>
       </c>
       <c r="E2" s="6">
-        <v>131</v>
+        <v>345.55532168052969</v>
       </c>
       <c r="F2" s="6">
-        <v>111</v>
+        <v>292.04998154935089</v>
       </c>
       <c r="G2" s="6">
-        <v>95</v>
+        <v>246.34750352063568</v>
       </c>
       <c r="H2" s="6">
-        <f t="shared" ref="H2:K6" si="0">D2*0.06</f>
         <v>8.58</v>
       </c>
       <c r="I2" s="6">
-        <f t="shared" si="0"/>
         <v>7.8599999999999994</v>
       </c>
       <c r="J2" s="6">
-        <f t="shared" si="0"/>
         <v>6.66</v>
       </c>
       <c r="K2" s="6">
-        <f t="shared" si="0"/>
         <v>5.7</v>
       </c>
       <c r="L2" s="6">
@@ -5512,21 +5563,21 @@
         <v>77.5</v>
       </c>
       <c r="O2" s="6">
-        <v>40.520000000000003</v>
+        <v>36.36</v>
       </c>
       <c r="P2" s="6">
-        <v>40.520000000000003</v>
+        <v>36.36</v>
       </c>
       <c r="Q2" s="6">
-        <v>40.520000000000003</v>
+        <v>36.36</v>
       </c>
       <c r="R2" s="6">
-        <v>40.520000000000003</v>
+        <v>36.36</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="B3" t="s">
         <v>62</v>
@@ -5535,31 +5586,27 @@
         <v>57</v>
       </c>
       <c r="D3" s="6">
-        <v>105</v>
+        <v>1047.8129109022511</v>
       </c>
       <c r="E3" s="6">
-        <v>100.8</v>
+        <v>978.70184656614526</v>
       </c>
       <c r="F3" s="6">
-        <v>92.4</v>
+        <v>824.87399368900628</v>
       </c>
       <c r="G3" s="6">
-        <v>84</v>
+        <v>695.5694217053242</v>
       </c>
       <c r="H3" s="6">
-        <f t="shared" si="0"/>
         <v>6.3</v>
       </c>
       <c r="I3" s="6">
-        <f t="shared" si="0"/>
         <v>6.048</v>
       </c>
       <c r="J3" s="6">
-        <f t="shared" si="0"/>
         <v>5.5440000000000005</v>
       </c>
       <c r="K3" s="6">
-        <f t="shared" si="0"/>
         <v>5.04</v>
       </c>
       <c r="L3" s="6">
@@ -5572,21 +5619,21 @@
         <v>92</v>
       </c>
       <c r="O3" s="6">
-        <v>40.520000000000003</v>
+        <v>38.36</v>
       </c>
       <c r="P3" s="6">
-        <v>40.520000000000003</v>
+        <v>38.36</v>
       </c>
       <c r="Q3" s="6">
-        <v>40.520000000000003</v>
+        <v>38.36</v>
       </c>
       <c r="R3" s="6">
-        <v>40.520000000000003</v>
+        <v>38.36</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="B4" t="s">
         <v>63</v>
@@ -5595,31 +5642,27 @@
         <v>57</v>
       </c>
       <c r="D4" s="6">
-        <v>36</v>
+        <v>339.98184875019854</v>
       </c>
       <c r="E4" s="6">
-        <v>34.6</v>
+        <v>317.68795702887405</v>
       </c>
       <c r="F4" s="6">
-        <v>31.7</v>
+        <v>267.52670065589393</v>
       </c>
       <c r="G4" s="6">
-        <v>28.8</v>
+        <v>226.28300097144361</v>
       </c>
       <c r="H4" s="6">
-        <f t="shared" si="0"/>
         <v>2.16</v>
       </c>
       <c r="I4" s="6">
-        <f t="shared" si="0"/>
         <v>2.0760000000000001</v>
       </c>
       <c r="J4" s="6">
-        <f t="shared" si="0"/>
         <v>1.9019999999999999</v>
       </c>
       <c r="K4" s="6">
-        <f t="shared" si="0"/>
         <v>1.728</v>
       </c>
       <c r="L4" s="6">
@@ -5632,21 +5675,21 @@
         <v>94.5</v>
       </c>
       <c r="O4" s="6">
-        <v>40.520000000000003</v>
+        <v>37.28</v>
       </c>
       <c r="P4" s="6">
-        <v>40.520000000000003</v>
+        <v>37.28</v>
       </c>
       <c r="Q4" s="6">
-        <v>40.520000000000003</v>
+        <v>37.28</v>
       </c>
       <c r="R4" s="6">
-        <v>40.520000000000003</v>
+        <v>37.28</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="B5" t="s">
         <v>64</v>
@@ -5655,31 +5698,27 @@
         <v>57</v>
       </c>
       <c r="D5" s="6">
-        <v>105</v>
+        <v>836.02093954966858</v>
       </c>
       <c r="E5" s="6">
-        <v>100.8</v>
+        <v>780.28621024635731</v>
       </c>
       <c r="F5" s="6">
-        <v>92.4</v>
+        <v>657.66980577907259</v>
       </c>
       <c r="G5" s="6">
-        <v>84</v>
+        <v>555.11790386097982</v>
       </c>
       <c r="H5" s="6">
-        <f t="shared" si="0"/>
         <v>6.3</v>
       </c>
       <c r="I5" s="6">
-        <f t="shared" si="0"/>
         <v>6.048</v>
       </c>
       <c r="J5" s="6">
-        <f t="shared" si="0"/>
         <v>5.5440000000000005</v>
       </c>
       <c r="K5" s="6">
-        <f t="shared" si="0"/>
         <v>5.04</v>
       </c>
       <c r="L5" s="6">
@@ -5692,16 +5731,16 @@
         <v>94.5</v>
       </c>
       <c r="O5" s="6">
-        <v>40.520000000000003</v>
+        <v>35.1</v>
       </c>
       <c r="P5" s="6">
-        <v>40.520000000000003</v>
+        <v>35.1</v>
       </c>
       <c r="Q5" s="6">
-        <v>40.520000000000003</v>
+        <v>35.1</v>
       </c>
       <c r="R5" s="6">
-        <v>40.520000000000003</v>
+        <v>35.1</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
@@ -5715,34 +5754,27 @@
         <v>57</v>
       </c>
       <c r="D6" s="6">
-        <v>85</v>
+        <v>947.49039815629101</v>
       </c>
       <c r="E6" s="6">
-        <f>D6*(1-0.075)</f>
-        <v>78.625</v>
+        <v>876.42861829456922</v>
       </c>
       <c r="F6" s="6">
-        <f>E6-(1-0.075)</f>
-        <v>77.7</v>
+        <v>866.11769337345663</v>
       </c>
       <c r="G6" s="6">
-        <f>F6-(1-0.075)</f>
-        <v>76.775000000000006</v>
+        <v>855.80676845234404</v>
       </c>
       <c r="H6" s="6">
-        <f t="shared" si="0"/>
         <v>5.0999999999999996</v>
       </c>
       <c r="I6" s="6">
-        <f t="shared" si="0"/>
         <v>4.7175000000000002</v>
       </c>
       <c r="J6" s="6">
-        <f t="shared" si="0"/>
         <v>4.6619999999999999</v>
       </c>
       <c r="K6" s="6">
-        <f t="shared" si="0"/>
         <v>4.6065000000000005</v>
       </c>
       <c r="L6" s="6">
@@ -5769,41 +5801,37 @@
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="B7" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="C7" t="s">
         <v>57</v>
       </c>
       <c r="D7" s="6">
-        <v>143</v>
+        <v>1047.8129109022511</v>
       </c>
       <c r="E7" s="6">
-        <v>131</v>
+        <v>978.70184656614526</v>
       </c>
       <c r="F7" s="6">
-        <v>111</v>
+        <v>824.87399368900628</v>
       </c>
       <c r="G7" s="6">
-        <v>95</v>
+        <v>695.5694217053242</v>
       </c>
       <c r="H7" s="6">
-        <f t="shared" ref="H7" si="1">D7*0.06</f>
-        <v>8.58</v>
+        <v>6.3</v>
       </c>
       <c r="I7" s="6">
-        <f t="shared" ref="I7" si="2">E7*0.06</f>
-        <v>7.8599999999999994</v>
+        <v>6.048</v>
       </c>
       <c r="J7" s="6">
-        <f t="shared" ref="J7" si="3">F7*0.06</f>
-        <v>6.66</v>
+        <v>5.5440000000000005</v>
       </c>
       <c r="K7" s="6">
-        <f t="shared" ref="K7" si="4">G7*0.06</f>
-        <v>5.7</v>
+        <v>5.04</v>
       </c>
       <c r="L7" s="6">
         <v>65</v>
@@ -5863,7 +5891,7 @@
         <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="C2" t="s">
         <v>61</v>
@@ -5871,11 +5899,11 @@
       <c r="D2">
         <v>0</v>
       </c>
-      <c r="E2" t="s">
-        <v>88</v>
+      <c r="E2">
+        <v>7650000</v>
       </c>
       <c r="F2">
-        <v>0.8</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -5883,19 +5911,19 @@
         <v>38</v>
       </c>
       <c r="B3" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="C3" t="s">
         <v>62</v>
       </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3" t="s">
-        <v>89</v>
+      <c r="D3" s="15">
+        <v>125000</v>
+      </c>
+      <c r="E3">
+        <v>112000</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -5903,7 +5931,7 @@
         <v>38</v>
       </c>
       <c r="B4" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="C4" t="s">
         <v>63</v>
@@ -5911,11 +5939,11 @@
       <c r="D4">
         <v>0</v>
       </c>
-      <c r="E4" t="s">
-        <v>90</v>
+      <c r="E4">
+        <v>2610000</v>
       </c>
       <c r="F4">
-        <v>0.75</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -5923,19 +5951,19 @@
         <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="C5" t="s">
         <v>64</v>
       </c>
-      <c r="D5">
-        <v>160000</v>
-      </c>
-      <c r="E5" t="s">
-        <v>91</v>
+      <c r="D5" s="14">
+        <v>910000</v>
+      </c>
+      <c r="E5">
+        <v>5400000</v>
       </c>
       <c r="F5">
-        <v>0.5</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -5948,14 +5976,14 @@
       <c r="C6" t="s">
         <v>65</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="15">
         <v>100000</v>
       </c>
-      <c r="E6" t="s">
-        <v>92</v>
+      <c r="E6">
+        <v>12950000</v>
       </c>
       <c r="F6">
-        <v>1.5</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -5963,19 +5991,19 @@
         <v>29</v>
       </c>
       <c r="B7" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="C7" t="s">
         <v>61</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="13">
         <v>400000</v>
       </c>
-      <c r="E7" t="s">
-        <v>93</v>
+      <c r="E7">
+        <v>400000</v>
       </c>
       <c r="F7">
-        <v>0.4</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -5983,7 +6011,7 @@
         <v>29</v>
       </c>
       <c r="B8" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="C8" t="s">
         <v>62</v>
@@ -5991,11 +6019,11 @@
       <c r="D8">
         <v>0</v>
       </c>
-      <c r="E8" t="s">
-        <v>94</v>
+      <c r="E8">
+        <v>260000</v>
       </c>
       <c r="F8">
-        <v>0.5</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -6003,7 +6031,7 @@
         <v>29</v>
       </c>
       <c r="B9" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="C9" t="s">
         <v>63</v>
@@ -6011,11 +6039,11 @@
       <c r="D9">
         <v>0</v>
       </c>
-      <c r="E9" t="s">
-        <v>94</v>
+      <c r="E9">
+        <v>200000</v>
       </c>
       <c r="F9">
-        <v>0.5</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -6023,7 +6051,7 @@
         <v>29</v>
       </c>
       <c r="B10" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="C10" t="s">
         <v>64</v>
@@ -6031,11 +6059,11 @@
       <c r="D10">
         <v>1700000</v>
       </c>
-      <c r="E10" t="s">
-        <v>90</v>
+      <c r="E10">
+        <v>500000</v>
       </c>
       <c r="F10">
-        <v>0.3</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -6051,11 +6079,11 @@
       <c r="D11">
         <v>0</v>
       </c>
-      <c r="E11" t="s">
-        <v>94</v>
+      <c r="E11">
+        <v>450000</v>
       </c>
       <c r="F11">
-        <v>0.6</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -6063,7 +6091,7 @@
         <v>30</v>
       </c>
       <c r="B12" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="C12" t="s">
         <v>61</v>
@@ -6071,11 +6099,11 @@
       <c r="D12">
         <v>0</v>
       </c>
-      <c r="E12" t="s">
-        <v>90</v>
+      <c r="E12">
+        <v>800000</v>
       </c>
       <c r="F12">
-        <v>0.8</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -6083,7 +6111,7 @@
         <v>30</v>
       </c>
       <c r="B13" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="C13" t="s">
         <v>62</v>
@@ -6091,11 +6119,11 @@
       <c r="D13">
         <v>0</v>
       </c>
-      <c r="E13" t="s">
-        <v>95</v>
+      <c r="E13">
+        <v>125000</v>
       </c>
       <c r="F13">
-        <v>1</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -6103,7 +6131,7 @@
         <v>30</v>
       </c>
       <c r="B14" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="C14" t="s">
         <v>63</v>
@@ -6111,11 +6139,11 @@
       <c r="D14">
         <v>0</v>
       </c>
-      <c r="E14" t="s">
-        <v>91</v>
+      <c r="E14">
+        <v>1000000</v>
       </c>
       <c r="F14">
-        <v>1</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -6123,7 +6151,7 @@
         <v>30</v>
       </c>
       <c r="B15" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="C15" t="s">
         <v>64</v>
@@ -6131,11 +6159,11 @@
       <c r="D15">
         <v>0</v>
       </c>
-      <c r="E15" t="s">
-        <v>96</v>
+      <c r="E15">
+        <v>1360000</v>
       </c>
       <c r="F15">
-        <v>0.9</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -6151,11 +6179,11 @@
       <c r="D16">
         <v>0</v>
       </c>
-      <c r="E16" t="s">
-        <v>97</v>
+      <c r="E16">
+        <v>10600000</v>
       </c>
       <c r="F16">
-        <v>1.2</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -6163,19 +6191,19 @@
         <v>38</v>
       </c>
       <c r="B17" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="C17" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="D17">
         <v>0</v>
       </c>
-      <c r="E17" t="s">
-        <v>95</v>
+      <c r="E17">
+        <v>6290000</v>
       </c>
       <c r="F17">
-        <v>0.5</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -6183,19 +6211,19 @@
         <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="C18" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="D18">
         <v>0</v>
       </c>
-      <c r="E18" t="s">
-        <v>94</v>
+      <c r="E18">
+        <v>2000000</v>
       </c>
       <c r="F18">
-        <v>0.5</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -6203,19 +6231,19 @@
         <v>30</v>
       </c>
       <c r="B19" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="C19" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="D19">
         <v>0</v>
       </c>
-      <c r="E19" t="s">
-        <v>95</v>
+      <c r="E19">
+        <v>11195000</v>
       </c>
       <c r="F19">
-        <v>0.5</v>
+        <v>0.02</v>
       </c>
     </row>
   </sheetData>
@@ -6226,6 +6254,1550 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5A2BEAB-012A-44FE-9D5A-F890D4AF74D1}">
+  <dimension ref="A1:S26"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C1" t="s">
+        <v>143</v>
+      </c>
+      <c r="D1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E1" t="s">
+        <v>145</v>
+      </c>
+      <c r="F1" t="s">
+        <v>146</v>
+      </c>
+      <c r="G1" t="s">
+        <v>147</v>
+      </c>
+      <c r="H1" t="s">
+        <v>148</v>
+      </c>
+      <c r="I1" t="s">
+        <v>149</v>
+      </c>
+      <c r="J1" t="s">
+        <v>150</v>
+      </c>
+      <c r="K1" t="s">
+        <v>151</v>
+      </c>
+      <c r="L1" t="s">
+        <v>152</v>
+      </c>
+      <c r="M1" t="s">
+        <v>153</v>
+      </c>
+      <c r="N1" t="s">
+        <v>154</v>
+      </c>
+      <c r="O1" t="s">
+        <v>155</v>
+      </c>
+      <c r="P1" t="s">
+        <v>156</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>157</v>
+      </c>
+      <c r="R1" t="s">
+        <v>158</v>
+      </c>
+      <c r="S1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2026</v>
+      </c>
+      <c r="B2">
+        <v>200000</v>
+      </c>
+      <c r="C2">
+        <v>800000</v>
+      </c>
+      <c r="D2">
+        <v>125000</v>
+      </c>
+      <c r="E2">
+        <v>631000</v>
+      </c>
+      <c r="F2">
+        <v>530000</v>
+      </c>
+      <c r="G2">
+        <v>3228000</v>
+      </c>
+      <c r="H2">
+        <v>400000</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>1700000</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
+      <c r="Q2">
+        <v>0</v>
+      </c>
+      <c r="R2">
+        <v>0</v>
+      </c>
+      <c r="S2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2027</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>2610000</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>1164000</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3">
+        <v>100000</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="P3">
+        <v>0</v>
+      </c>
+      <c r="Q3">
+        <v>0</v>
+      </c>
+      <c r="R3">
+        <v>5300000</v>
+      </c>
+      <c r="S3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2028</v>
+      </c>
+      <c r="B4">
+        <v>2176000</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>4500000</v>
+      </c>
+      <c r="F4">
+        <v>1993000</v>
+      </c>
+      <c r="G4">
+        <v>1000000</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>260000</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>100000</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>3718000</v>
+      </c>
+      <c r="R4">
+        <v>10600000</v>
+      </c>
+      <c r="S4">
+        <v>1360000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2029</v>
+      </c>
+      <c r="B5">
+        <v>7459000</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>112000</v>
+      </c>
+      <c r="E5">
+        <v>3188000</v>
+      </c>
+      <c r="F5">
+        <v>1160000</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>350000</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <v>800000</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>2270000</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2030</v>
+      </c>
+      <c r="B6">
+        <v>7650000</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>6290000</v>
+      </c>
+      <c r="F6">
+        <v>12950000</v>
+      </c>
+      <c r="G6">
+        <v>5400000</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>450000</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>1000000</v>
+      </c>
+      <c r="P6">
+        <v>0</v>
+      </c>
+      <c r="Q6">
+        <v>11195000</v>
+      </c>
+      <c r="R6">
+        <v>10000000</v>
+      </c>
+      <c r="S6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2031</v>
+      </c>
+      <c r="B7">
+        <v>4600000</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>1700000</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>740000</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>2000000</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7">
+        <v>0</v>
+      </c>
+      <c r="P7">
+        <v>0</v>
+      </c>
+      <c r="Q7">
+        <v>0</v>
+      </c>
+      <c r="R7">
+        <v>0</v>
+      </c>
+      <c r="S7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>2032</v>
+      </c>
+      <c r="B8">
+        <v>5415000</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>2000000</v>
+      </c>
+      <c r="F8">
+        <v>3500000</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8">
+        <v>0</v>
+      </c>
+      <c r="N8">
+        <v>540000</v>
+      </c>
+      <c r="O8">
+        <v>0</v>
+      </c>
+      <c r="P8">
+        <v>0</v>
+      </c>
+      <c r="Q8">
+        <v>890000</v>
+      </c>
+      <c r="R8">
+        <v>0</v>
+      </c>
+      <c r="S8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>2033</v>
+      </c>
+      <c r="B9">
+        <v>600000</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="L9">
+        <v>0</v>
+      </c>
+      <c r="M9">
+        <v>0</v>
+      </c>
+      <c r="N9">
+        <v>0</v>
+      </c>
+      <c r="O9">
+        <v>0</v>
+      </c>
+      <c r="P9">
+        <v>0</v>
+      </c>
+      <c r="Q9">
+        <v>0</v>
+      </c>
+      <c r="R9">
+        <v>6700000</v>
+      </c>
+      <c r="S9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>2034</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10">
+        <v>0</v>
+      </c>
+      <c r="N10">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>0</v>
+      </c>
+      <c r="P10">
+        <v>0</v>
+      </c>
+      <c r="Q10">
+        <v>0</v>
+      </c>
+      <c r="R10">
+        <v>5600000</v>
+      </c>
+      <c r="S10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A11" s="16">
+        <v>2035</v>
+      </c>
+      <c r="B11" s="16">
+        <v>0</v>
+      </c>
+      <c r="C11" s="16">
+        <v>0</v>
+      </c>
+      <c r="D11" s="16">
+        <v>0</v>
+      </c>
+      <c r="E11" s="16">
+        <v>0</v>
+      </c>
+      <c r="F11" s="16">
+        <v>0</v>
+      </c>
+      <c r="G11" s="16">
+        <v>0</v>
+      </c>
+      <c r="H11" s="16">
+        <v>0</v>
+      </c>
+      <c r="I11" s="16">
+        <v>0</v>
+      </c>
+      <c r="J11" s="16">
+        <v>0</v>
+      </c>
+      <c r="K11" s="16">
+        <v>150000</v>
+      </c>
+      <c r="L11" s="16">
+        <v>270000</v>
+      </c>
+      <c r="M11" s="16">
+        <v>0</v>
+      </c>
+      <c r="N11" s="16">
+        <v>0</v>
+      </c>
+      <c r="O11" s="16">
+        <v>0</v>
+      </c>
+      <c r="P11" s="16">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="16">
+        <v>1500000</v>
+      </c>
+      <c r="R11" s="16">
+        <v>1870000</v>
+      </c>
+      <c r="S11" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>2036</v>
+      </c>
+      <c r="B12">
+        <v>7650000</v>
+      </c>
+      <c r="C12">
+        <v>2610000</v>
+      </c>
+      <c r="D12">
+        <v>112000</v>
+      </c>
+      <c r="E12">
+        <v>6290000</v>
+      </c>
+      <c r="F12">
+        <v>12950000</v>
+      </c>
+      <c r="G12">
+        <v>5400000</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>260000</v>
+      </c>
+      <c r="K12">
+        <v>2000000</v>
+      </c>
+      <c r="L12">
+        <v>450000</v>
+      </c>
+      <c r="M12">
+        <v>0</v>
+      </c>
+      <c r="N12">
+        <v>800000</v>
+      </c>
+      <c r="O12">
+        <v>1000000</v>
+      </c>
+      <c r="P12">
+        <v>0</v>
+      </c>
+      <c r="Q12">
+        <v>11195000</v>
+      </c>
+      <c r="R12">
+        <v>10600000</v>
+      </c>
+      <c r="S12">
+        <v>1360000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>2037</v>
+      </c>
+      <c r="B13">
+        <v>7650000</v>
+      </c>
+      <c r="C13">
+        <v>2610000</v>
+      </c>
+      <c r="D13">
+        <v>112000</v>
+      </c>
+      <c r="E13">
+        <v>6290000</v>
+      </c>
+      <c r="F13">
+        <v>12950000</v>
+      </c>
+      <c r="G13">
+        <v>5400000</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>260000</v>
+      </c>
+      <c r="K13">
+        <v>2000000</v>
+      </c>
+      <c r="L13">
+        <v>450000</v>
+      </c>
+      <c r="M13">
+        <v>0</v>
+      </c>
+      <c r="N13">
+        <v>800000</v>
+      </c>
+      <c r="O13">
+        <v>1000000</v>
+      </c>
+      <c r="P13">
+        <v>0</v>
+      </c>
+      <c r="Q13">
+        <v>11195000</v>
+      </c>
+      <c r="R13">
+        <v>10600000</v>
+      </c>
+      <c r="S13">
+        <v>1360000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>2038</v>
+      </c>
+      <c r="B14">
+        <v>7650000</v>
+      </c>
+      <c r="C14">
+        <v>2610000</v>
+      </c>
+      <c r="D14">
+        <v>112000</v>
+      </c>
+      <c r="E14">
+        <v>6290000</v>
+      </c>
+      <c r="F14">
+        <v>12950000</v>
+      </c>
+      <c r="G14">
+        <v>5400000</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>260000</v>
+      </c>
+      <c r="K14">
+        <v>2000000</v>
+      </c>
+      <c r="L14">
+        <v>450000</v>
+      </c>
+      <c r="M14">
+        <v>0</v>
+      </c>
+      <c r="N14">
+        <v>800000</v>
+      </c>
+      <c r="O14">
+        <v>1000000</v>
+      </c>
+      <c r="P14">
+        <v>0</v>
+      </c>
+      <c r="Q14">
+        <v>11195000</v>
+      </c>
+      <c r="R14">
+        <v>10600000</v>
+      </c>
+      <c r="S14">
+        <v>1360000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>2039</v>
+      </c>
+      <c r="B15">
+        <v>7650000</v>
+      </c>
+      <c r="C15">
+        <v>2610000</v>
+      </c>
+      <c r="D15">
+        <v>112000</v>
+      </c>
+      <c r="E15">
+        <v>6290000</v>
+      </c>
+      <c r="F15">
+        <v>12950000</v>
+      </c>
+      <c r="G15">
+        <v>5400000</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>260000</v>
+      </c>
+      <c r="K15">
+        <v>2000000</v>
+      </c>
+      <c r="L15">
+        <v>450000</v>
+      </c>
+      <c r="M15">
+        <v>0</v>
+      </c>
+      <c r="N15">
+        <v>800000</v>
+      </c>
+      <c r="O15">
+        <v>1000000</v>
+      </c>
+      <c r="P15">
+        <v>0</v>
+      </c>
+      <c r="Q15">
+        <v>11195000</v>
+      </c>
+      <c r="R15">
+        <v>10600000</v>
+      </c>
+      <c r="S15">
+        <v>1360000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>2040</v>
+      </c>
+      <c r="B16">
+        <v>7650000</v>
+      </c>
+      <c r="C16">
+        <v>2610000</v>
+      </c>
+      <c r="D16">
+        <v>112000</v>
+      </c>
+      <c r="E16">
+        <v>6290000</v>
+      </c>
+      <c r="F16">
+        <v>12950000</v>
+      </c>
+      <c r="G16">
+        <v>5400000</v>
+      </c>
+      <c r="H16">
+        <v>0</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>260000</v>
+      </c>
+      <c r="K16">
+        <v>2000000</v>
+      </c>
+      <c r="L16">
+        <v>450000</v>
+      </c>
+      <c r="M16">
+        <v>0</v>
+      </c>
+      <c r="N16">
+        <v>800000</v>
+      </c>
+      <c r="O16">
+        <v>1000000</v>
+      </c>
+      <c r="P16">
+        <v>0</v>
+      </c>
+      <c r="Q16">
+        <v>11195000</v>
+      </c>
+      <c r="R16">
+        <v>10600000</v>
+      </c>
+      <c r="S16">
+        <v>1360000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>2041</v>
+      </c>
+      <c r="B17">
+        <v>7650000</v>
+      </c>
+      <c r="C17">
+        <v>2610000</v>
+      </c>
+      <c r="D17">
+        <v>112000</v>
+      </c>
+      <c r="E17">
+        <v>6290000</v>
+      </c>
+      <c r="F17">
+        <v>12950000</v>
+      </c>
+      <c r="G17">
+        <v>5400000</v>
+      </c>
+      <c r="H17">
+        <v>0</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>260000</v>
+      </c>
+      <c r="K17">
+        <v>2000000</v>
+      </c>
+      <c r="L17">
+        <v>450000</v>
+      </c>
+      <c r="M17">
+        <v>0</v>
+      </c>
+      <c r="N17">
+        <v>800000</v>
+      </c>
+      <c r="O17">
+        <v>1000000</v>
+      </c>
+      <c r="P17">
+        <v>0</v>
+      </c>
+      <c r="Q17">
+        <v>11195000</v>
+      </c>
+      <c r="R17">
+        <v>10600000</v>
+      </c>
+      <c r="S17">
+        <v>1360000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>2042</v>
+      </c>
+      <c r="B18">
+        <v>7650000</v>
+      </c>
+      <c r="C18">
+        <v>2610000</v>
+      </c>
+      <c r="D18">
+        <v>112000</v>
+      </c>
+      <c r="E18">
+        <v>6290000</v>
+      </c>
+      <c r="F18">
+        <v>12950000</v>
+      </c>
+      <c r="G18">
+        <v>5400000</v>
+      </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>260000</v>
+      </c>
+      <c r="K18">
+        <v>2000000</v>
+      </c>
+      <c r="L18">
+        <v>450000</v>
+      </c>
+      <c r="M18">
+        <v>0</v>
+      </c>
+      <c r="N18">
+        <v>800000</v>
+      </c>
+      <c r="O18">
+        <v>1000000</v>
+      </c>
+      <c r="P18">
+        <v>0</v>
+      </c>
+      <c r="Q18">
+        <v>11195000</v>
+      </c>
+      <c r="R18">
+        <v>10600000</v>
+      </c>
+      <c r="S18">
+        <v>1360000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>2043</v>
+      </c>
+      <c r="B19">
+        <v>7650000</v>
+      </c>
+      <c r="C19">
+        <v>2610000</v>
+      </c>
+      <c r="D19">
+        <v>112000</v>
+      </c>
+      <c r="E19">
+        <v>6290000</v>
+      </c>
+      <c r="F19">
+        <v>12950000</v>
+      </c>
+      <c r="G19">
+        <v>5400000</v>
+      </c>
+      <c r="H19">
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <v>260000</v>
+      </c>
+      <c r="K19">
+        <v>2000000</v>
+      </c>
+      <c r="L19">
+        <v>450000</v>
+      </c>
+      <c r="M19">
+        <v>0</v>
+      </c>
+      <c r="N19">
+        <v>800000</v>
+      </c>
+      <c r="O19">
+        <v>1000000</v>
+      </c>
+      <c r="P19">
+        <v>0</v>
+      </c>
+      <c r="Q19">
+        <v>11195000</v>
+      </c>
+      <c r="R19">
+        <v>10600000</v>
+      </c>
+      <c r="S19">
+        <v>1360000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>2044</v>
+      </c>
+      <c r="B20">
+        <v>7650000</v>
+      </c>
+      <c r="C20">
+        <v>2610000</v>
+      </c>
+      <c r="D20">
+        <v>112000</v>
+      </c>
+      <c r="E20">
+        <v>6290000</v>
+      </c>
+      <c r="F20">
+        <v>12950000</v>
+      </c>
+      <c r="G20">
+        <v>5400000</v>
+      </c>
+      <c r="H20">
+        <v>0</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>260000</v>
+      </c>
+      <c r="K20">
+        <v>2000000</v>
+      </c>
+      <c r="L20">
+        <v>450000</v>
+      </c>
+      <c r="M20">
+        <v>0</v>
+      </c>
+      <c r="N20">
+        <v>800000</v>
+      </c>
+      <c r="O20">
+        <v>1000000</v>
+      </c>
+      <c r="P20">
+        <v>0</v>
+      </c>
+      <c r="Q20">
+        <v>11195000</v>
+      </c>
+      <c r="R20">
+        <v>10600000</v>
+      </c>
+      <c r="S20">
+        <v>1360000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>2045</v>
+      </c>
+      <c r="B21">
+        <v>7650000</v>
+      </c>
+      <c r="C21">
+        <v>2610000</v>
+      </c>
+      <c r="D21">
+        <v>112000</v>
+      </c>
+      <c r="E21">
+        <v>6290000</v>
+      </c>
+      <c r="F21">
+        <v>12950000</v>
+      </c>
+      <c r="G21">
+        <v>5400000</v>
+      </c>
+      <c r="H21">
+        <v>0</v>
+      </c>
+      <c r="I21">
+        <v>0</v>
+      </c>
+      <c r="J21">
+        <v>260000</v>
+      </c>
+      <c r="K21">
+        <v>2000000</v>
+      </c>
+      <c r="L21">
+        <v>450000</v>
+      </c>
+      <c r="M21">
+        <v>0</v>
+      </c>
+      <c r="N21">
+        <v>800000</v>
+      </c>
+      <c r="O21">
+        <v>1000000</v>
+      </c>
+      <c r="P21">
+        <v>0</v>
+      </c>
+      <c r="Q21">
+        <v>11195000</v>
+      </c>
+      <c r="R21">
+        <v>10600000</v>
+      </c>
+      <c r="S21">
+        <v>1360000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>2046</v>
+      </c>
+      <c r="B22">
+        <v>7650000</v>
+      </c>
+      <c r="C22">
+        <v>2610000</v>
+      </c>
+      <c r="D22">
+        <v>112000</v>
+      </c>
+      <c r="E22">
+        <v>6290000</v>
+      </c>
+      <c r="F22">
+        <v>12950000</v>
+      </c>
+      <c r="G22">
+        <v>5400000</v>
+      </c>
+      <c r="H22">
+        <v>0</v>
+      </c>
+      <c r="I22">
+        <v>0</v>
+      </c>
+      <c r="J22">
+        <v>260000</v>
+      </c>
+      <c r="K22">
+        <v>2000000</v>
+      </c>
+      <c r="L22">
+        <v>450000</v>
+      </c>
+      <c r="M22">
+        <v>0</v>
+      </c>
+      <c r="N22">
+        <v>800000</v>
+      </c>
+      <c r="O22">
+        <v>1000000</v>
+      </c>
+      <c r="P22">
+        <v>0</v>
+      </c>
+      <c r="Q22">
+        <v>11195000</v>
+      </c>
+      <c r="R22">
+        <v>10600000</v>
+      </c>
+      <c r="S22">
+        <v>1360000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>2047</v>
+      </c>
+      <c r="B23">
+        <v>7650000</v>
+      </c>
+      <c r="C23">
+        <v>2610000</v>
+      </c>
+      <c r="D23">
+        <v>112000</v>
+      </c>
+      <c r="E23">
+        <v>6290000</v>
+      </c>
+      <c r="F23">
+        <v>12950000</v>
+      </c>
+      <c r="G23">
+        <v>5400000</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>260000</v>
+      </c>
+      <c r="K23">
+        <v>2000000</v>
+      </c>
+      <c r="L23">
+        <v>450000</v>
+      </c>
+      <c r="M23">
+        <v>0</v>
+      </c>
+      <c r="N23">
+        <v>800000</v>
+      </c>
+      <c r="O23">
+        <v>1000000</v>
+      </c>
+      <c r="P23">
+        <v>0</v>
+      </c>
+      <c r="Q23">
+        <v>11195000</v>
+      </c>
+      <c r="R23">
+        <v>10600000</v>
+      </c>
+      <c r="S23">
+        <v>1360000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>2048</v>
+      </c>
+      <c r="B24">
+        <v>7650000</v>
+      </c>
+      <c r="C24">
+        <v>2610000</v>
+      </c>
+      <c r="D24">
+        <v>112000</v>
+      </c>
+      <c r="E24">
+        <v>6290000</v>
+      </c>
+      <c r="F24">
+        <v>12950000</v>
+      </c>
+      <c r="G24">
+        <v>5400000</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>260000</v>
+      </c>
+      <c r="K24">
+        <v>2000000</v>
+      </c>
+      <c r="L24">
+        <v>450000</v>
+      </c>
+      <c r="M24">
+        <v>0</v>
+      </c>
+      <c r="N24">
+        <v>800000</v>
+      </c>
+      <c r="O24">
+        <v>1000000</v>
+      </c>
+      <c r="P24">
+        <v>0</v>
+      </c>
+      <c r="Q24">
+        <v>11195000</v>
+      </c>
+      <c r="R24">
+        <v>10600000</v>
+      </c>
+      <c r="S24">
+        <v>1360000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>2049</v>
+      </c>
+      <c r="B25">
+        <v>7650000</v>
+      </c>
+      <c r="C25">
+        <v>2610000</v>
+      </c>
+      <c r="D25">
+        <v>112000</v>
+      </c>
+      <c r="E25">
+        <v>6290000</v>
+      </c>
+      <c r="F25">
+        <v>12950000</v>
+      </c>
+      <c r="G25">
+        <v>5400000</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <v>260000</v>
+      </c>
+      <c r="K25">
+        <v>2000000</v>
+      </c>
+      <c r="L25">
+        <v>450000</v>
+      </c>
+      <c r="M25">
+        <v>0</v>
+      </c>
+      <c r="N25">
+        <v>800000</v>
+      </c>
+      <c r="O25">
+        <v>1000000</v>
+      </c>
+      <c r="P25">
+        <v>0</v>
+      </c>
+      <c r="Q25">
+        <v>11195000</v>
+      </c>
+      <c r="R25">
+        <v>10600000</v>
+      </c>
+      <c r="S25">
+        <v>1360000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>2050</v>
+      </c>
+      <c r="B26">
+        <v>7650000</v>
+      </c>
+      <c r="C26">
+        <v>2610000</v>
+      </c>
+      <c r="D26">
+        <v>112000</v>
+      </c>
+      <c r="E26">
+        <v>6290000</v>
+      </c>
+      <c r="F26">
+        <v>12950000</v>
+      </c>
+      <c r="G26">
+        <v>5400000</v>
+      </c>
+      <c r="H26">
+        <v>0</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>260000</v>
+      </c>
+      <c r="K26">
+        <v>2000000</v>
+      </c>
+      <c r="L26">
+        <v>450000</v>
+      </c>
+      <c r="M26">
+        <v>0</v>
+      </c>
+      <c r="N26">
+        <v>800000</v>
+      </c>
+      <c r="O26">
+        <v>1000000</v>
+      </c>
+      <c r="P26">
+        <v>0</v>
+      </c>
+      <c r="Q26">
+        <v>11195000</v>
+      </c>
+      <c r="R26">
+        <v>10600000</v>
+      </c>
+      <c r="S26">
+        <v>1360000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F3C079C-E0FE-4643-9E48-5AE3F12A3520}">
   <dimension ref="A1:E217"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9925,7 +11497,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E6FE4EC-E3E7-42F5-A9DB-0136E2BCE431}">
   <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -10053,7 +11625,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7E57138-F43E-470A-BCDF-3CE08782F05D}">
   <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>